<commit_message>
feat: complete engineering forms and acceptance refinements
</commit_message>
<xml_diff>
--- a/templates/excel/form_2_5_V1.xlsx
+++ b/templates/excel/form_2_5_V1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\gitProject\YindaSurveySystem\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C266B318-BA8B-487E-9C10-4CB2D1072722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD69E627-9856-40B6-8865-002475903D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
-  <si>
-    <t>附表2.5    隧洞工程状况调查表</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
   <si>
     <t>处</t>
   </si>
@@ -212,6 +209,13 @@
   </si>
   <si>
     <t>注：洞身包括洞身衬砌层、围岩等。</t>
+  </si>
+  <si>
+    <t>附表2.5</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">    隧洞工程状况调查表</t>
   </si>
 </sst>
 </file>
@@ -304,23 +308,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -549,18 +553,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.35" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
+      <c r="A1" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:10" ht="7.2" customHeight="1">
       <c r="A2" s="1"/>
@@ -577,22 +583,22 @@
     <row r="3" spans="1:10" ht="17.55" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="J3" s="4"/>
     </row>
@@ -609,101 +615,101 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>6</v>
+      <c r="A5" s="5" t="s">
+        <v>5</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="6" t="s">
-        <v>7</v>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="6"/>
-    </row>
-    <row r="6" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="5"/>
+      <c r="E7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="5"/>
+      <c r="G7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="5"/>
+      <c r="I7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A8" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
-      <c r="D8" s="6" t="s">
-        <v>20</v>
+      <c r="D8" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="7"/>
-      <c r="J8" s="6"/>
-    </row>
-    <row r="9" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="9"/>
+      <c r="E9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>25</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>26</v>
       </c>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
@@ -712,249 +718,249 @@
     </row>
     <row r="10" spans="1:10" ht="33.6" customHeight="1">
       <c r="A10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="5">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="6">
-        <v>1</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" spans="1:10" ht="28.8" customHeight="1">
       <c r="A11" s="7"/>
-      <c r="B11" s="6">
+      <c r="B11" s="5">
         <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="27.15" customHeight="1">
       <c r="A12" s="7"/>
-      <c r="B12" s="6">
+      <c r="B12" s="5">
         <v>3</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="28.8" customHeight="1">
       <c r="A13" s="7"/>
-      <c r="B13" s="6">
+      <c r="B13" s="5">
         <v>4</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="1:10" ht="35.25" customHeight="1">
       <c r="A14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="6">
-        <v>1</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
     </row>
     <row r="15" spans="1:10" ht="44.85" customHeight="1">
       <c r="A15" s="7"/>
-      <c r="B15" s="6">
+      <c r="B15" s="5">
         <v>2</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" spans="1:10" ht="70.349999999999994" customHeight="1">
       <c r="A16" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="5">
+        <v>1</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="6">
-        <v>1</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" ht="40.049999999999997" customHeight="1">
       <c r="A17" s="7"/>
-      <c r="B17" s="6">
+      <c r="B17" s="5">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="7"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10" ht="35.25" customHeight="1">
       <c r="A18" s="7"/>
-      <c r="B18" s="6">
+      <c r="B18" s="5">
         <v>3</v>
       </c>
       <c r="C18" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" spans="1:10" ht="30.45" customHeight="1">
       <c r="A19" s="7"/>
-      <c r="B19" s="6">
+      <c r="B19" s="5">
         <v>4</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" s="7"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8" customHeight="1">
       <c r="A20" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="5">
+        <v>1</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="6">
-        <v>1</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="33.6" customHeight="1">
       <c r="A21" s="7"/>
-      <c r="B21" s="6">
+      <c r="B21" s="5">
         <v>2</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="7"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="27.15" customHeight="1">
       <c r="A22" s="7"/>
-      <c r="B22" s="6">
+      <c r="B22" s="5">
         <v>3</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="23" spans="1:10" ht="22.35" customHeight="1">
       <c r="A23" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -963,49 +969,84 @@
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J23" s="5"/>
+    </row>
+    <row r="24" spans="1:10" ht="20.85" customHeight="1">
+      <c r="A24" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J23" s="6"/>
-    </row>
-    <row r="24" spans="1:10" ht="20.85" customHeight="1">
-      <c r="A24" s="6" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="5"/>
+      <c r="E24" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="5"/>
+      <c r="G24" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6" t="s">
+      <c r="H24" s="5"/>
+      <c r="I24" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6" t="s">
+      <c r="J24" s="5"/>
+    </row>
+    <row r="25" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A25" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="J24" s="6"/>
-    </row>
-    <row r="25" spans="1:10" ht="19.2" customHeight="1">
-      <c r="A25" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="42">
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:J9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:J11"/>
+    <mergeCell ref="F12:J12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="F15:J15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F18:J18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="F19:J19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C12:D12"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="C23:H23"/>
     <mergeCell ref="A25:J25"/>
@@ -1013,40 +1054,6 @@
     <mergeCell ref="F21:J21"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="F22:J22"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="F18:J18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="F19:J19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="F20:J20"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:J15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:J17"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:J14"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:J9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="H8:I8"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>